<commit_message>
assumptions for CE mid and high scenarios
</commit_message>
<xml_diff>
--- a/aluminium/inputs/10 regions Al data.xlsx
+++ b/aluminium/inputs/10 regions Al data.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\damamahou\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\omnia_demand_industry\aluminium\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFD6C4D2-C3D2-42D8-A6F9-DF7AE049AEE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{411738A5-39A3-4DEB-A931-F9408A5C428A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-1540" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4890" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="baseline" sheetId="1" r:id="rId1"/>
     <sheet name="recycling rate scenario" sheetId="2" r:id="rId2"/>
     <sheet name="lifetime scenario" sheetId="4" r:id="rId3"/>
+    <sheet name="CE Mid High" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="24">
   <si>
     <t>China</t>
   </si>
@@ -87,12 +88,39 @@
   <si>
     <t>Based on BAU scenarios, lifetime gradually increase and reach their target values by 2050 in each region.</t>
   </si>
+  <si>
+    <t>Global</t>
+  </si>
+  <si>
+    <t>I would consider this to be the Medium scenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://international-aluminium.org/wp-content/uploads/2022/09/Making-1.5-Aligned-Aluminium-possible.pdf </t>
+  </si>
+  <si>
+    <t>Hence:</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>For a high scenario, I'd consider 16.7% total global production reduction, as suggested by this ref:</t>
+  </si>
+  <si>
+    <t>16.7% is obtained from point 6 at page 15: "Without any action, aluminium demand is expected to rise 80% by 2050. Material efficiency can play a critical role in ensuring that aluminium is used effectively, potentially reducing demand by 29 Mt and limiting growth to 50%."</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -116,6 +144,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -134,16 +185,38 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -422,46 +495,46 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AU28"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.9296875" customWidth="1"/>
-    <col min="3" max="3" width="13.19921875" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="13.53125" customWidth="1"/>
-    <col min="6" max="6" width="9.9296875" customWidth="1"/>
-    <col min="7" max="7" width="18.19921875" customWidth="1"/>
-    <col min="8" max="8" width="11.796875" customWidth="1"/>
-    <col min="9" max="9" width="6.9296875" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="18.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="9" max="9" width="7" customWidth="1"/>
     <col min="10" max="10" width="8" customWidth="1"/>
-    <col min="11" max="11" width="13.796875" customWidth="1"/>
-    <col min="12" max="12" width="9.73046875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.53125" customWidth="1"/>
-    <col min="15" max="15" width="12.73046875" customWidth="1"/>
-    <col min="17" max="17" width="13.19921875" customWidth="1"/>
-    <col min="18" max="18" width="10.73046875" customWidth="1"/>
-    <col min="19" max="19" width="18.73046875" customWidth="1"/>
-    <col min="20" max="20" width="13.06640625" customWidth="1"/>
-    <col min="23" max="23" width="12.73046875" customWidth="1"/>
-    <col min="24" max="24" width="9.73046875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="19.3984375" customWidth="1"/>
-    <col min="27" max="27" width="14.33203125" customWidth="1"/>
-    <col min="29" max="29" width="13.06640625" customWidth="1"/>
+    <col min="11" max="11" width="13.85546875" customWidth="1"/>
+    <col min="12" max="12" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.5703125" customWidth="1"/>
+    <col min="15" max="15" width="12.7109375" customWidth="1"/>
+    <col min="17" max="17" width="13.140625" customWidth="1"/>
+    <col min="18" max="18" width="10.7109375" customWidth="1"/>
+    <col min="19" max="19" width="18.7109375" customWidth="1"/>
+    <col min="20" max="20" width="13" customWidth="1"/>
+    <col min="23" max="23" width="12.7109375" customWidth="1"/>
+    <col min="24" max="24" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="19.42578125" customWidth="1"/>
+    <col min="27" max="27" width="14.28515625" customWidth="1"/>
+    <col min="29" max="29" width="13" customWidth="1"/>
     <col min="30" max="30" width="11" customWidth="1"/>
-    <col min="31" max="31" width="19.3984375" customWidth="1"/>
-    <col min="32" max="32" width="11.1328125" customWidth="1"/>
+    <col min="31" max="31" width="19.42578125" customWidth="1"/>
+    <col min="32" max="32" width="11.140625" customWidth="1"/>
     <col min="35" max="35" width="13" customWidth="1"/>
-    <col min="36" max="36" width="9.73046875" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="10.3984375" customWidth="1"/>
-    <col min="39" max="39" width="13.3984375" customWidth="1"/>
-    <col min="41" max="41" width="14.46484375" customWidth="1"/>
-    <col min="42" max="42" width="10.33203125" customWidth="1"/>
-    <col min="43" max="43" width="14.19921875" customWidth="1"/>
-    <col min="44" max="44" width="11.59765625" customWidth="1"/>
-    <col min="47" max="47" width="13.86328125" customWidth="1"/>
-    <col min="48" max="48" width="9.73046875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="10.42578125" customWidth="1"/>
+    <col min="39" max="39" width="13.42578125" customWidth="1"/>
+    <col min="41" max="41" width="14.42578125" customWidth="1"/>
+    <col min="42" max="42" width="10.28515625" customWidth="1"/>
+    <col min="43" max="43" width="14.140625" customWidth="1"/>
+    <col min="44" max="44" width="11.5703125" customWidth="1"/>
+    <col min="47" max="47" width="13.85546875" customWidth="1"/>
+    <col min="48" max="48" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -595,7 +668,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -729,7 +802,7 @@
         <v>1521.85860557879</v>
       </c>
     </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -863,7 +936,7 @@
         <v>1825.8742046659579</v>
       </c>
     </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -997,7 +1070,7 @@
         <v>2054.4106704007022</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2027</v>
       </c>
@@ -1131,7 +1204,7 @@
         <v>2276.464463624633</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2028</v>
       </c>
@@ -1265,7 +1338,7 @@
         <v>2494.0954045426361</v>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2029</v>
       </c>
@@ -1399,7 +1472,7 @@
         <v>2711.1774140437728</v>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2030</v>
       </c>
@@ -1533,7 +1606,7 @@
         <v>2928.9661701862842</v>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2031</v>
       </c>
@@ -1667,7 +1740,7 @@
         <v>3147.1996183589749</v>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2032</v>
       </c>
@@ -1801,7 +1874,7 @@
         <v>3364.0686030843922</v>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2033</v>
       </c>
@@ -1935,7 +2008,7 @@
         <v>3576.7519911959539</v>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2034</v>
       </c>
@@ -2069,7 +2142,7 @@
         <v>3782.3099873235719</v>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2035</v>
       </c>
@@ -2203,7 +2276,7 @@
         <v>3978.9873032455448</v>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2036</v>
       </c>
@@ -2337,7 +2410,7 @@
         <v>4167.7196744564644</v>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2037</v>
       </c>
@@ -2471,7 +2544,7 @@
         <v>4352.2247732213109</v>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2038</v>
       </c>
@@ -2605,7 +2678,7 @@
         <v>4538.8511500759123</v>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2039</v>
       </c>
@@ -2739,7 +2812,7 @@
         <v>4735.7175104024682</v>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2040</v>
       </c>
@@ -2873,7 +2946,7 @@
         <v>4949.9830062979563</v>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2041</v>
       </c>
@@ -3007,7 +3080,7 @@
         <v>5185.9504227679126</v>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2042</v>
       </c>
@@ -3141,7 +3214,7 @@
         <v>5446.1700108725199</v>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2043</v>
       </c>
@@ -3275,7 +3348,7 @@
         <v>5731.1045962553226</v>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2044</v>
       </c>
@@ -3409,7 +3482,7 @@
         <v>6037.8864119556511</v>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2045</v>
       </c>
@@ -3543,7 +3616,7 @@
         <v>6362.2344476877424</v>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2046</v>
       </c>
@@ -3677,7 +3750,7 @@
         <v>6700.4429753337918</v>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2047</v>
       </c>
@@ -3811,7 +3884,7 @@
         <v>7048.5298708808796</v>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2048</v>
       </c>
@@ -3945,7 +4018,7 @@
         <v>7403.5487787357233</v>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2049</v>
       </c>
@@ -4079,7 +4152,7 @@
         <v>7763.7963839380282</v>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2050</v>
       </c>
@@ -4221,42 +4294,42 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF956376-06A0-42E5-ADBD-08A2C76D85B4}">
   <dimension ref="A1:AW28"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="13.9296875" customWidth="1"/>
-    <col min="5" max="5" width="13.19921875" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="13.53125" customWidth="1"/>
-    <col min="8" max="8" width="9.9296875" customWidth="1"/>
-    <col min="9" max="9" width="18.19921875" customWidth="1"/>
-    <col min="10" max="10" width="11.796875" customWidth="1"/>
-    <col min="11" max="11" width="6.9296875" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="7" customWidth="1"/>
     <col min="12" max="12" width="8" customWidth="1"/>
-    <col min="13" max="13" width="13.796875" customWidth="1"/>
-    <col min="15" max="15" width="18.53125" customWidth="1"/>
-    <col min="17" max="17" width="12.73046875" customWidth="1"/>
-    <col min="19" max="19" width="13.19921875" customWidth="1"/>
-    <col min="20" max="20" width="10.73046875" customWidth="1"/>
-    <col min="21" max="21" width="18.73046875" customWidth="1"/>
-    <col min="22" max="22" width="13.06640625" customWidth="1"/>
-    <col min="25" max="25" width="12.73046875" customWidth="1"/>
-    <col min="27" max="27" width="19.3984375" customWidth="1"/>
-    <col min="29" max="29" width="14.33203125" customWidth="1"/>
-    <col min="31" max="31" width="13.06640625" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" customWidth="1"/>
+    <col min="15" max="15" width="18.5703125" customWidth="1"/>
+    <col min="17" max="17" width="12.7109375" customWidth="1"/>
+    <col min="19" max="19" width="13.140625" customWidth="1"/>
+    <col min="20" max="20" width="10.7109375" customWidth="1"/>
+    <col min="21" max="21" width="18.7109375" customWidth="1"/>
+    <col min="22" max="22" width="13" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" customWidth="1"/>
+    <col min="27" max="27" width="19.42578125" customWidth="1"/>
+    <col min="29" max="29" width="14.28515625" customWidth="1"/>
+    <col min="31" max="31" width="13" customWidth="1"/>
     <col min="32" max="32" width="11" customWidth="1"/>
-    <col min="33" max="33" width="19.3984375" customWidth="1"/>
-    <col min="34" max="34" width="11.1328125" customWidth="1"/>
+    <col min="33" max="33" width="19.42578125" customWidth="1"/>
+    <col min="34" max="34" width="11.140625" customWidth="1"/>
     <col min="37" max="37" width="13" customWidth="1"/>
-    <col min="39" max="39" width="10.3984375" customWidth="1"/>
-    <col min="41" max="41" width="13.3984375" customWidth="1"/>
-    <col min="43" max="43" width="14.46484375" customWidth="1"/>
-    <col min="44" max="44" width="10.33203125" customWidth="1"/>
-    <col min="45" max="45" width="14.19921875" customWidth="1"/>
-    <col min="46" max="46" width="11.59765625" customWidth="1"/>
-    <col min="49" max="49" width="13.86328125" customWidth="1"/>
+    <col min="39" max="39" width="10.42578125" customWidth="1"/>
+    <col min="41" max="41" width="13.42578125" customWidth="1"/>
+    <col min="43" max="43" width="14.42578125" customWidth="1"/>
+    <col min="44" max="44" width="10.28515625" customWidth="1"/>
+    <col min="45" max="45" width="14.140625" customWidth="1"/>
+    <col min="46" max="46" width="11.5703125" customWidth="1"/>
+    <col min="49" max="49" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C1" s="1" t="s">
         <v>10</v>
       </c>
@@ -4390,7 +4463,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>14</v>
       </c>
@@ -4527,7 +4600,7 @@
         <v>1535.9096538483</v>
       </c>
     </row>
-    <row r="3" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C3">
         <v>2025</v>
       </c>
@@ -4661,7 +4734,7 @@
         <v>1856.949492015935</v>
       </c>
     </row>
-    <row r="4" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C4">
         <v>2026</v>
       </c>
@@ -4795,7 +4868,7 @@
         <v>2108.4496156756359</v>
       </c>
     </row>
-    <row r="5" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C5">
         <v>2027</v>
       </c>
@@ -4929,7 +5002,7 @@
         <v>2358.0155413296479</v>
       </c>
     </row>
-    <row r="6" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C6">
         <v>2028</v>
       </c>
@@ -5063,7 +5136,7 @@
         <v>2607.5438178580512</v>
       </c>
     </row>
-    <row r="7" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C7">
         <v>2029</v>
       </c>
@@ -5197,7 +5270,7 @@
         <v>2860.9174991461582</v>
       </c>
     </row>
-    <row r="8" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C8">
         <v>2030</v>
       </c>
@@ -5331,7 +5404,7 @@
         <v>3119.413208170502</v>
       </c>
     </row>
-    <row r="9" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C9">
         <v>2031</v>
       </c>
@@ -5465,7 +5538,7 @@
         <v>3382.6829318317232</v>
       </c>
     </row>
-    <row r="10" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C10">
         <v>2032</v>
       </c>
@@ -5599,7 +5672,7 @@
         <v>3648.6349101532378</v>
       </c>
     </row>
-    <row r="11" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C11">
         <v>2033</v>
       </c>
@@ -5733,7 +5806,7 @@
         <v>3913.9588178163222</v>
       </c>
     </row>
-    <row r="12" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C12">
         <v>2034</v>
       </c>
@@ -5867,7 +5940,7 @@
         <v>4175.1226208054741</v>
       </c>
     </row>
-    <row r="13" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C13">
         <v>2035</v>
       </c>
@@ -6001,7 +6074,7 @@
         <v>4429.8894204865774</v>
       </c>
     </row>
-    <row r="14" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C14">
         <v>2036</v>
       </c>
@@ -6135,7 +6208,7 @@
         <v>4679.09290372535</v>
       </c>
     </row>
-    <row r="15" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C15">
         <v>2037</v>
       </c>
@@ -6269,7 +6342,7 @@
         <v>4926.9576448872413</v>
       </c>
     </row>
-    <row r="16" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C16">
         <v>2038</v>
       </c>
@@ -6403,7 +6476,7 @@
         <v>5181.0045415454451</v>
       </c>
     </row>
-    <row r="17" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="17" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C17">
         <v>2039</v>
       </c>
@@ -6537,7 +6610,7 @@
         <v>5451.0542369248178</v>
       </c>
     </row>
-    <row r="18" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="18" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C18">
         <v>2040</v>
       </c>
@@ -6671,7 +6744,7 @@
         <v>5746.2256145248393</v>
       </c>
     </row>
-    <row r="19" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="19" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C19">
         <v>2041</v>
       </c>
@@ -6805,7 +6878,7 @@
         <v>6072.6741633541087</v>
       </c>
     </row>
-    <row r="20" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="20" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C20">
         <v>2042</v>
       </c>
@@ -6939,7 +7012,7 @@
         <v>6434.3703494159163</v>
       </c>
     </row>
-    <row r="21" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="21" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C21">
         <v>2043</v>
       </c>
@@ -7073,7 +7146,7 @@
         <v>6832.6635165501029</v>
       </c>
     </row>
-    <row r="22" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="22" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C22">
         <v>2044</v>
       </c>
@@ -7207,7 +7280,7 @@
         <v>7265.0603467848014</v>
       </c>
     </row>
-    <row r="23" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="23" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C23">
         <v>2045</v>
       </c>
@@ -7341,7 +7414,7 @@
         <v>7727.1688140232463</v>
       </c>
     </row>
-    <row r="24" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="24" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C24">
         <v>2046</v>
       </c>
@@ -7475,7 +7548,7 @@
         <v>8214.8438570653198</v>
       </c>
     </row>
-    <row r="25" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="25" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C25">
         <v>2047</v>
       </c>
@@ -7609,7 +7682,7 @@
         <v>8723.5857569817072</v>
       </c>
     </row>
-    <row r="26" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="26" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C26">
         <v>2048</v>
       </c>
@@ -7743,7 +7816,7 @@
         <v>9249.974512773033</v>
       </c>
     </row>
-    <row r="27" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="27" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C27">
         <v>2049</v>
       </c>
@@ -7877,7 +7950,7 @@
         <v>9792.0062046110452</v>
       </c>
     </row>
-    <row r="28" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="28" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C28">
         <v>2050</v>
       </c>
@@ -8019,42 +8092,42 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6984D29-3D0B-4159-95BC-BC1D39185047}">
   <dimension ref="A1:AW28"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="13.9296875" customWidth="1"/>
-    <col min="5" max="5" width="13.19921875" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="13.53125" customWidth="1"/>
-    <col min="8" max="8" width="9.9296875" customWidth="1"/>
-    <col min="9" max="9" width="18.19921875" customWidth="1"/>
-    <col min="10" max="10" width="11.796875" customWidth="1"/>
-    <col min="11" max="11" width="6.9296875" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="7" customWidth="1"/>
     <col min="12" max="12" width="8" customWidth="1"/>
-    <col min="13" max="13" width="13.796875" customWidth="1"/>
-    <col min="15" max="15" width="18.53125" customWidth="1"/>
-    <col min="17" max="17" width="12.73046875" customWidth="1"/>
-    <col min="19" max="19" width="13.19921875" customWidth="1"/>
-    <col min="20" max="20" width="10.73046875" customWidth="1"/>
-    <col min="21" max="21" width="18.73046875" customWidth="1"/>
-    <col min="22" max="22" width="13.06640625" customWidth="1"/>
-    <col min="25" max="25" width="12.73046875" customWidth="1"/>
-    <col min="27" max="27" width="19.3984375" customWidth="1"/>
-    <col min="29" max="29" width="14.33203125" customWidth="1"/>
-    <col min="31" max="31" width="13.06640625" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" customWidth="1"/>
+    <col min="15" max="15" width="18.5703125" customWidth="1"/>
+    <col min="17" max="17" width="12.7109375" customWidth="1"/>
+    <col min="19" max="19" width="13.140625" customWidth="1"/>
+    <col min="20" max="20" width="10.7109375" customWidth="1"/>
+    <col min="21" max="21" width="18.7109375" customWidth="1"/>
+    <col min="22" max="22" width="13" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" customWidth="1"/>
+    <col min="27" max="27" width="19.42578125" customWidth="1"/>
+    <col min="29" max="29" width="14.28515625" customWidth="1"/>
+    <col min="31" max="31" width="13" customWidth="1"/>
     <col min="32" max="32" width="11" customWidth="1"/>
-    <col min="33" max="33" width="19.3984375" customWidth="1"/>
-    <col min="34" max="34" width="11.1328125" customWidth="1"/>
+    <col min="33" max="33" width="19.42578125" customWidth="1"/>
+    <col min="34" max="34" width="11.140625" customWidth="1"/>
     <col min="37" max="37" width="13" customWidth="1"/>
-    <col min="39" max="39" width="10.3984375" customWidth="1"/>
-    <col min="41" max="41" width="13.3984375" customWidth="1"/>
-    <col min="43" max="43" width="14.46484375" customWidth="1"/>
-    <col min="44" max="44" width="10.33203125" customWidth="1"/>
-    <col min="45" max="45" width="14.19921875" customWidth="1"/>
-    <col min="46" max="46" width="11.59765625" customWidth="1"/>
-    <col min="49" max="49" width="13.86328125" customWidth="1"/>
+    <col min="39" max="39" width="10.42578125" customWidth="1"/>
+    <col min="41" max="41" width="13.42578125" customWidth="1"/>
+    <col min="43" max="43" width="14.42578125" customWidth="1"/>
+    <col min="44" max="44" width="10.28515625" customWidth="1"/>
+    <col min="45" max="45" width="14.140625" customWidth="1"/>
+    <col min="46" max="46" width="11.5703125" customWidth="1"/>
+    <col min="49" max="49" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C1" s="1" t="s">
         <v>10</v>
       </c>
@@ -8188,7 +8261,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
@@ -8325,7 +8398,7 @@
         <v>1521.85860557879</v>
       </c>
     </row>
-    <row r="3" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C3">
         <v>2025</v>
       </c>
@@ -8459,7 +8532,7 @@
         <v>1825.841551135725</v>
       </c>
     </row>
-    <row r="4" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C4">
         <v>2026</v>
       </c>
@@ -8593,7 +8666,7 @@
         <v>2054.280318888962</v>
       </c>
     </row>
-    <row r="5" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C5">
         <v>2027</v>
       </c>
@@ -8727,7 +8800,7 @@
         <v>2276.0771223694942</v>
       </c>
     </row>
-    <row r="6" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C6">
         <v>2028</v>
       </c>
@@ -8861,7 +8934,7 @@
         <v>2493.1203307904229</v>
       </c>
     </row>
-    <row r="7" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C7">
         <v>2029</v>
       </c>
@@ -8995,7 +9068,7 @@
         <v>2708.9982965097061</v>
       </c>
     </row>
-    <row r="8" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C8">
         <v>2030</v>
       </c>
@@ -9129,7 +9202,7 @@
         <v>2924.550752128001</v>
       </c>
     </row>
-    <row r="9" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C9">
         <v>2031</v>
       </c>
@@ -9263,7 +9336,7 @@
         <v>3138.9896324621091</v>
       </c>
     </row>
-    <row r="10" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C10">
         <v>2032</v>
       </c>
@@ -9397,7 +9470,7 @@
         <v>3349.9274638410479</v>
       </c>
     </row>
-    <row r="11" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C11">
         <v>2033</v>
       </c>
@@ -9531,7 +9604,7 @@
         <v>3553.9781439038902</v>
       </c>
     </row>
-    <row r="12" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C12">
         <v>2034</v>
       </c>
@@ -9665,7 +9738,7 @@
         <v>3747.67617182089</v>
       </c>
     </row>
-    <row r="13" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C13">
         <v>2035</v>
       </c>
@@ -9799,7 +9872,7 @@
         <v>3928.740476389547</v>
       </c>
     </row>
-    <row r="14" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C14">
         <v>2036</v>
       </c>
@@ -9933,7 +10006,7 @@
         <v>4097.5070941897029</v>
       </c>
     </row>
-    <row r="15" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C15">
         <v>2037</v>
       </c>
@@ -10067,7 +10140,7 @@
         <v>4256.986790355958</v>
       </c>
     </row>
-    <row r="16" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:49" x14ac:dyDescent="0.25">
       <c r="C16">
         <v>2038</v>
       </c>
@@ -10201,7 +10274,7 @@
         <v>4412.7832118863043</v>
       </c>
     </row>
-    <row r="17" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="17" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C17">
         <v>2039</v>
       </c>
@@ -10335,7 +10408,7 @@
         <v>4572.3979915283398</v>
       </c>
     </row>
-    <row r="18" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="18" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C18">
         <v>2040</v>
       </c>
@@ -10469,7 +10542,7 @@
         <v>4742.6897877473066</v>
       </c>
     </row>
-    <row r="19" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="19" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C19">
         <v>2041</v>
       </c>
@@ -10603,7 +10676,7 @@
         <v>4928.0990577412003</v>
       </c>
     </row>
-    <row r="20" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="20" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C20">
         <v>2042</v>
       </c>
@@ -10737,7 +10810,7 @@
         <v>5131.7527886158896</v>
       </c>
     </row>
-    <row r="21" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="21" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C21">
         <v>2043</v>
       </c>
@@ -10871,7 +10944,7 @@
         <v>5355.0103304922068</v>
       </c>
     </row>
-    <row r="22" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="22" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C22">
         <v>2044</v>
       </c>
@@ -11005,7 +11078,7 @@
         <v>5596.0218346837682</v>
       </c>
     </row>
-    <row r="23" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="23" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C23">
         <v>2045</v>
       </c>
@@ -11139,7 +11212,7 @@
         <v>5851.4239248707536</v>
       </c>
     </row>
-    <row r="24" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="24" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C24">
         <v>2046</v>
       </c>
@@ -11273,7 +11346,7 @@
         <v>6118.1356279966913</v>
       </c>
     </row>
-    <row r="25" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="25" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C25">
         <v>2047</v>
       </c>
@@ -11407,7 +11480,7 @@
         <v>6392.3862662038482</v>
       </c>
     </row>
-    <row r="26" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="26" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C26">
         <v>2048</v>
       </c>
@@ -11541,7 +11614,7 @@
         <v>6671.0065361479647</v>
       </c>
     </row>
-    <row r="27" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="27" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C27">
         <v>2049</v>
       </c>
@@ -11675,7 +11748,7 @@
         <v>6951.7133851920862</v>
       </c>
     </row>
-    <row r="28" spans="3:49" x14ac:dyDescent="0.45">
+    <row r="28" spans="3:49" x14ac:dyDescent="0.25">
       <c r="C28">
         <v>2050</v>
       </c>
@@ -11812,4 +11885,1635 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EBC7690-7AE8-4B19-95C9-8DFAEBAA00F1}">
+  <dimension ref="B2:S29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="18" max="18" width="11.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:18" ht="45" x14ac:dyDescent="0.25">
+      <c r="C2" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="R2" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B3" s="5">
+        <v>2024</v>
+      </c>
+      <c r="C3" s="3">
+        <f>1-('lifetime scenario'!D2/baseline!B2)</f>
+        <v>0</v>
+      </c>
+      <c r="D3" s="3">
+        <f>1-('lifetime scenario'!E2/baseline!C2)</f>
+        <v>0</v>
+      </c>
+      <c r="E3" s="3">
+        <f>1-('lifetime scenario'!F2/baseline!D2)</f>
+        <v>0</v>
+      </c>
+      <c r="F3" s="3">
+        <f>1-('lifetime scenario'!G2/baseline!E2)</f>
+        <v>0</v>
+      </c>
+      <c r="G3" s="3">
+        <f>1-('lifetime scenario'!H2/baseline!F2)</f>
+        <v>0</v>
+      </c>
+      <c r="H3" s="3">
+        <f>1-('lifetime scenario'!I2/baseline!G2)</f>
+        <v>0</v>
+      </c>
+      <c r="I3" s="3">
+        <f>1-('lifetime scenario'!J2/baseline!H2)</f>
+        <v>0</v>
+      </c>
+      <c r="J3" s="3">
+        <f>1-('lifetime scenario'!K2/baseline!I2)</f>
+        <v>0</v>
+      </c>
+      <c r="K3" s="3">
+        <f>1-('lifetime scenario'!L2/baseline!J2)</f>
+        <v>0</v>
+      </c>
+      <c r="L3" s="3">
+        <f>1-('lifetime scenario'!M2/baseline!K2)</f>
+        <v>0</v>
+      </c>
+      <c r="N3" s="5">
+        <v>2024</v>
+      </c>
+      <c r="O3" s="3">
+        <f>1-SUM('lifetime scenario'!D2:M2)/SUM(baseline!B2:K2)</f>
+        <v>0</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>2019</v>
+      </c>
+      <c r="R3" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B4" s="5">
+        <v>2025</v>
+      </c>
+      <c r="C4" s="3">
+        <f>1-('lifetime scenario'!D3/baseline!B3)</f>
+        <v>1.0549294706230228E-5</v>
+      </c>
+      <c r="D4" s="3">
+        <f>1-('lifetime scenario'!E3/baseline!C3)</f>
+        <v>7.4213561783720294E-6</v>
+      </c>
+      <c r="E4" s="3">
+        <f>1-('lifetime scenario'!F3/baseline!D3)</f>
+        <v>8.035472359613216E-6</v>
+      </c>
+      <c r="F4" s="3">
+        <f>1-('lifetime scenario'!G3/baseline!E3)</f>
+        <v>8.8214592601776332E-6</v>
+      </c>
+      <c r="G4" s="3">
+        <f>1-('lifetime scenario'!H3/baseline!F3)</f>
+        <v>7.1587959064034479E-6</v>
+      </c>
+      <c r="H4" s="3">
+        <f>1-('lifetime scenario'!I3/baseline!G3)</f>
+        <v>6.1272695051073356E-6</v>
+      </c>
+      <c r="I4" s="3">
+        <f>1-('lifetime scenario'!J3/baseline!H3)</f>
+        <v>7.7311212013375652E-6</v>
+      </c>
+      <c r="J4" s="3">
+        <f>1-('lifetime scenario'!K3/baseline!I3)</f>
+        <v>4.5856099455399146E-6</v>
+      </c>
+      <c r="K4" s="3">
+        <f>1-('lifetime scenario'!L3/baseline!J3)</f>
+        <v>6.9692643855923109E-6</v>
+      </c>
+      <c r="L4" s="3">
+        <f>1-('lifetime scenario'!M3/baseline!K3)</f>
+        <v>9.1387182656887944E-6</v>
+      </c>
+      <c r="N4" s="5">
+        <v>2025</v>
+      </c>
+      <c r="O4" s="3">
+        <f>1-SUM('lifetime scenario'!D3:M3)/SUM(baseline!B3:K3)</f>
+        <v>8.856151468505935E-6</v>
+      </c>
+      <c r="Q4" s="5">
+        <v>2023</v>
+      </c>
+      <c r="R4" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B5" s="5">
+        <v>2026</v>
+      </c>
+      <c r="C5" s="3">
+        <f>1-('lifetime scenario'!D4/baseline!B4)</f>
+        <v>5.0893982443289687E-5</v>
+      </c>
+      <c r="D5" s="3">
+        <f>1-('lifetime scenario'!E4/baseline!C4)</f>
+        <v>3.137472098191374E-5</v>
+      </c>
+      <c r="E5" s="3">
+        <f>1-('lifetime scenario'!F4/baseline!D4)</f>
+        <v>3.1725784195857365E-5</v>
+      </c>
+      <c r="F5" s="3">
+        <f>1-('lifetime scenario'!G4/baseline!E4)</f>
+        <v>3.9668996669961487E-5</v>
+      </c>
+      <c r="G5" s="3">
+        <f>1-('lifetime scenario'!H4/baseline!F4)</f>
+        <v>3.1583129978640656E-5</v>
+      </c>
+      <c r="H5" s="3">
+        <f>1-('lifetime scenario'!I4/baseline!G4)</f>
+        <v>3.1965968330327499E-5</v>
+      </c>
+      <c r="I5" s="3">
+        <f>1-('lifetime scenario'!J4/baseline!H4)</f>
+        <v>3.9902106822142791E-5</v>
+      </c>
+      <c r="J5" s="3">
+        <f>1-('lifetime scenario'!K4/baseline!I4)</f>
+        <v>2.156306641343253E-5</v>
+      </c>
+      <c r="K5" s="3">
+        <f>1-('lifetime scenario'!L4/baseline!J4)</f>
+        <v>3.1994013467429028E-5</v>
+      </c>
+      <c r="L5" s="3">
+        <f>1-('lifetime scenario'!M4/baseline!K4)</f>
+        <v>3.1833178944729035E-5</v>
+      </c>
+      <c r="N5" s="5">
+        <v>2026</v>
+      </c>
+      <c r="O5" s="3">
+        <f>1-SUM('lifetime scenario'!D4:M4)/SUM(baseline!B4:K4)</f>
+        <v>4.0050414420123026E-5</v>
+      </c>
+      <c r="Q5" s="5">
+        <v>2025</v>
+      </c>
+      <c r="R5" s="4">
+        <f>O4</f>
+        <v>8.856151468505935E-6</v>
+      </c>
+    </row>
+    <row r="6" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B6" s="5">
+        <v>2027</v>
+      </c>
+      <c r="C6" s="3">
+        <f>1-('lifetime scenario'!D5/baseline!B5)</f>
+        <v>1.652502133923095E-4</v>
+      </c>
+      <c r="D6" s="3">
+        <f>1-('lifetime scenario'!E5/baseline!C5)</f>
+        <v>8.9251740496565368E-5</v>
+      </c>
+      <c r="E6" s="3">
+        <f>1-('lifetime scenario'!F5/baseline!D5)</f>
+        <v>8.9945246172229432E-5</v>
+      </c>
+      <c r="F6" s="3">
+        <f>1-('lifetime scenario'!G5/baseline!E5)</f>
+        <v>1.2003876403599012E-4</v>
+      </c>
+      <c r="G6" s="3">
+        <f>1-('lifetime scenario'!H5/baseline!F5)</f>
+        <v>9.3404160652399426E-5</v>
+      </c>
+      <c r="H6" s="3">
+        <f>1-('lifetime scenario'!I5/baseline!G5)</f>
+        <v>1.0259757685027182E-4</v>
+      </c>
+      <c r="I6" s="3">
+        <f>1-('lifetime scenario'!J5/baseline!H5)</f>
+        <v>1.2660475346926159E-4</v>
+      </c>
+      <c r="J6" s="3">
+        <f>1-('lifetime scenario'!K5/baseline!I5)</f>
+        <v>6.4341240242793418E-5</v>
+      </c>
+      <c r="K6" s="3">
+        <f>1-('lifetime scenario'!L5/baseline!J5)</f>
+        <v>9.2708601997282258E-5</v>
+      </c>
+      <c r="L6" s="3">
+        <f>1-('lifetime scenario'!M5/baseline!K5)</f>
+        <v>8.4714874032609799E-5</v>
+      </c>
+      <c r="N6" s="5">
+        <v>2027</v>
+      </c>
+      <c r="O6" s="3">
+        <f>1-SUM('lifetime scenario'!D5:M5)/SUM(baseline!B5:K5)</f>
+        <v>1.2305015709535017E-4</v>
+      </c>
+      <c r="Q6" s="5">
+        <v>2030</v>
+      </c>
+      <c r="R6" s="4">
+        <f>O9</f>
+        <v>1.3763782578244399E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B7" s="5">
+        <v>2028</v>
+      </c>
+      <c r="C7" s="3">
+        <f>1-('lifetime scenario'!D6/baseline!B6)</f>
+        <v>4.3985275382563138E-4</v>
+      </c>
+      <c r="D7" s="3">
+        <f>1-('lifetime scenario'!E6/baseline!C6)</f>
+        <v>2.1053923057434698E-4</v>
+      </c>
+      <c r="E7" s="3">
+        <f>1-('lifetime scenario'!F6/baseline!D6)</f>
+        <v>2.1219004727002222E-4</v>
+      </c>
+      <c r="F7" s="3">
+        <f>1-('lifetime scenario'!G6/baseline!E6)</f>
+        <v>2.9923521444175094E-4</v>
+      </c>
+      <c r="G7" s="3">
+        <f>1-('lifetime scenario'!H6/baseline!F6)</f>
+        <v>2.2735917119143245E-4</v>
+      </c>
+      <c r="H7" s="3">
+        <f>1-('lifetime scenario'!I6/baseline!G6)</f>
+        <v>2.679888050528545E-4</v>
+      </c>
+      <c r="I7" s="3">
+        <f>1-('lifetime scenario'!J6/baseline!H6)</f>
+        <v>3.2494943043648306E-4</v>
+      </c>
+      <c r="J7" s="3">
+        <f>1-('lifetime scenario'!K6/baseline!I6)</f>
+        <v>1.5761981282524928E-4</v>
+      </c>
+      <c r="K7" s="3">
+        <f>1-('lifetime scenario'!L6/baseline!J6)</f>
+        <v>2.2067791111257673E-4</v>
+      </c>
+      <c r="L7" s="3">
+        <f>1-('lifetime scenario'!M6/baseline!K6)</f>
+        <v>1.9363229452218356E-4</v>
+      </c>
+      <c r="N7" s="5">
+        <v>2028</v>
+      </c>
+      <c r="O7" s="3">
+        <f>1-SUM('lifetime scenario'!D6:M6)/SUM(baseline!B6:K6)</f>
+        <v>3.1141560291592096E-4</v>
+      </c>
+      <c r="Q7" s="5">
+        <v>2035</v>
+      </c>
+      <c r="R7" s="4">
+        <f>O14</f>
+        <v>1.322158521410377E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B8" s="5">
+        <v>2029</v>
+      </c>
+      <c r="C8" s="3">
+        <f>1-('lifetime scenario'!D7/baseline!B7)</f>
+        <v>1.0167324869335692E-3</v>
+      </c>
+      <c r="D8" s="3">
+        <f>1-('lifetime scenario'!E7/baseline!C7)</f>
+        <v>4.4261129859435311E-4</v>
+      </c>
+      <c r="E8" s="3">
+        <f>1-('lifetime scenario'!F7/baseline!D7)</f>
+        <v>4.4815779215467977E-4</v>
+      </c>
+      <c r="F8" s="3">
+        <f>1-('lifetime scenario'!G7/baseline!E7)</f>
+        <v>6.5515771845514603E-4</v>
+      </c>
+      <c r="G8" s="3">
+        <f>1-('lifetime scenario'!H7/baseline!F7)</f>
+        <v>4.8624300044830537E-4</v>
+      </c>
+      <c r="H8" s="3">
+        <f>1-('lifetime scenario'!I7/baseline!G7)</f>
+        <v>6.1032830159335472E-4</v>
+      </c>
+      <c r="I8" s="3">
+        <f>1-('lifetime scenario'!J7/baseline!H7)</f>
+        <v>7.2924111090022503E-4</v>
+      </c>
+      <c r="J8" s="3">
+        <f>1-('lifetime scenario'!K7/baseline!I7)</f>
+        <v>3.4226953463123433E-4</v>
+      </c>
+      <c r="K8" s="3">
+        <f>1-('lifetime scenario'!L7/baseline!J7)</f>
+        <v>4.6794645465275675E-4</v>
+      </c>
+      <c r="L8" s="3">
+        <f>1-('lifetime scenario'!M7/baseline!K7)</f>
+        <v>3.9651414755115244E-4</v>
+      </c>
+      <c r="N8" s="5">
+        <v>2029</v>
+      </c>
+      <c r="O8" s="3">
+        <f>1-SUM('lifetime scenario'!D7:M7)/SUM(baseline!B7:K7)</f>
+        <v>6.9054069783314187E-4</v>
+      </c>
+      <c r="Q8" s="5">
+        <v>2040</v>
+      </c>
+      <c r="R8" s="4">
+        <f>O19</f>
+        <v>3.9106839655486669E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B9" s="5">
+        <v>2030</v>
+      </c>
+      <c r="C9" s="3">
+        <f>1-('lifetime scenario'!D8/baseline!B8)</f>
+        <v>2.093513454474949E-3</v>
+      </c>
+      <c r="D9" s="3">
+        <f>1-('lifetime scenario'!E8/baseline!C8)</f>
+        <v>8.5456441026188212E-4</v>
+      </c>
+      <c r="E9" s="3">
+        <f>1-('lifetime scenario'!F8/baseline!D8)</f>
+        <v>8.6839701558871774E-4</v>
+      </c>
+      <c r="F9" s="3">
+        <f>1-('lifetime scenario'!G8/baseline!E8)</f>
+        <v>1.2949208169720228E-3</v>
+      </c>
+      <c r="G9" s="3">
+        <f>1-('lifetime scenario'!H8/baseline!F8)</f>
+        <v>9.3951680606130239E-4</v>
+      </c>
+      <c r="H9" s="3">
+        <f>1-('lifetime scenario'!I8/baseline!G8)</f>
+        <v>1.248584748812176E-3</v>
+      </c>
+      <c r="I9" s="3">
+        <f>1-('lifetime scenario'!J8/baseline!H8)</f>
+        <v>1.4771488447223868E-3</v>
+      </c>
+      <c r="J9" s="3">
+        <f>1-('lifetime scenario'!K8/baseline!I8)</f>
+        <v>6.8043561702313404E-4</v>
+      </c>
+      <c r="K9" s="3">
+        <f>1-('lifetime scenario'!L8/baseline!J8)</f>
+        <v>9.0828088673933216E-4</v>
+      </c>
+      <c r="L9" s="3">
+        <f>1-('lifetime scenario'!M8/baseline!K8)</f>
+        <v>7.4238201133369763E-4</v>
+      </c>
+      <c r="N9" s="5">
+        <v>2030</v>
+      </c>
+      <c r="O9" s="3">
+        <f>1-SUM('lifetime scenario'!D8:M8)/SUM(baseline!B8:K8)</f>
+        <v>1.3763782578244399E-3</v>
+      </c>
+      <c r="Q9" s="5">
+        <v>2045</v>
+      </c>
+      <c r="R9" s="4">
+        <f>O24</f>
+        <v>7.1177024926353694E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B10" s="5">
+        <v>2031</v>
+      </c>
+      <c r="C10" s="3">
+        <f>1-('lifetime scenario'!D9/baseline!B9)</f>
+        <v>3.8986107766666445E-3</v>
+      </c>
+      <c r="D10" s="3">
+        <f>1-('lifetime scenario'!E9/baseline!C9)</f>
+        <v>1.5363026419739079E-3</v>
+      </c>
+      <c r="E10" s="3">
+        <f>1-('lifetime scenario'!F9/baseline!D9)</f>
+        <v>1.5654594883512951E-3</v>
+      </c>
+      <c r="F10" s="3">
+        <f>1-('lifetime scenario'!G9/baseline!E9)</f>
+        <v>2.3468880368955336E-3</v>
+      </c>
+      <c r="G10" s="3">
+        <f>1-('lifetime scenario'!H9/baseline!F9)</f>
+        <v>1.6660634314790146E-3</v>
+      </c>
+      <c r="H10" s="3">
+        <f>1-('lifetime scenario'!I9/baseline!G9)</f>
+        <v>2.3280632723484684E-3</v>
+      </c>
+      <c r="I10" s="3">
+        <f>1-('lifetime scenario'!J9/baseline!H9)</f>
+        <v>2.7357258521036876E-3</v>
+      </c>
+      <c r="J10" s="3">
+        <f>1-('lifetime scenario'!K9/baseline!I9)</f>
+        <v>1.2578607087783134E-3</v>
+      </c>
+      <c r="K10" s="3">
+        <f>1-('lifetime scenario'!L9/baseline!J9)</f>
+        <v>1.6441670403292141E-3</v>
+      </c>
+      <c r="L10" s="3">
+        <f>1-('lifetime scenario'!M9/baseline!K9)</f>
+        <v>1.2856749209793072E-3</v>
+      </c>
+      <c r="N10" s="5">
+        <v>2031</v>
+      </c>
+      <c r="O10" s="3">
+        <f>1-SUM('lifetime scenario'!D9:M9)/SUM(baseline!B9:K9)</f>
+        <v>2.5018115636511462E-3</v>
+      </c>
+      <c r="Q10" s="7">
+        <v>2050</v>
+      </c>
+      <c r="R10" s="4">
+        <f>O29</f>
+        <v>0.10326126048032036</v>
+      </c>
+    </row>
+    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B11" s="5">
+        <v>2032</v>
+      </c>
+      <c r="C11" s="3">
+        <f>1-('lifetime scenario'!D10/baseline!B10)</f>
+        <v>6.6394484489316064E-3</v>
+      </c>
+      <c r="D11" s="3">
+        <f>1-('lifetime scenario'!E10/baseline!C10)</f>
+        <v>2.597853315105203E-3</v>
+      </c>
+      <c r="E11" s="3">
+        <f>1-('lifetime scenario'!F10/baseline!D10)</f>
+        <v>2.6458930880305376E-3</v>
+      </c>
+      <c r="F11" s="3">
+        <f>1-('lifetime scenario'!G10/baseline!E10)</f>
+        <v>3.9410133958122096E-3</v>
+      </c>
+      <c r="G11" s="3">
+        <f>1-('lifetime scenario'!H10/baseline!F10)</f>
+        <v>2.7418341525303758E-3</v>
+      </c>
+      <c r="H11" s="3">
+        <f>1-('lifetime scenario'!I10/baseline!G10)</f>
+        <v>3.9918701993536532E-3</v>
+      </c>
+      <c r="I11" s="3">
+        <f>1-('lifetime scenario'!J10/baseline!H10)</f>
+        <v>4.6753986572296569E-3</v>
+      </c>
+      <c r="J11" s="3">
+        <f>1-('lifetime scenario'!K10/baseline!I10)</f>
+        <v>2.1793322576928453E-3</v>
+      </c>
+      <c r="K11" s="3">
+        <f>1-('lifetime scenario'!L10/baseline!J10)</f>
+        <v>2.8010046606582462E-3</v>
+      </c>
+      <c r="L11" s="3">
+        <f>1-('lifetime scenario'!M10/baseline!K10)</f>
+        <v>2.0783673979322126E-3</v>
+      </c>
+      <c r="N11" s="5">
+        <v>2032</v>
+      </c>
+      <c r="O11" s="3">
+        <f>1-SUM('lifetime scenario'!D10:M10)/SUM(baseline!B10:K10)</f>
+        <v>4.1905878761223647E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B12" s="5">
+        <v>2033</v>
+      </c>
+      <c r="C12" s="3">
+        <f>1-('lifetime scenario'!D11/baseline!B11)</f>
+        <v>1.0441068815112753E-2</v>
+      </c>
+      <c r="D12" s="3">
+        <f>1-('lifetime scenario'!E11/baseline!C11)</f>
+        <v>4.1583929598889569E-3</v>
+      </c>
+      <c r="E12" s="3">
+        <f>1-('lifetime scenario'!F11/baseline!D11)</f>
+        <v>4.2198386232860097E-3</v>
+      </c>
+      <c r="F12" s="3">
+        <f>1-('lifetime scenario'!G11/baseline!E11)</f>
+        <v>6.1861315348477053E-3</v>
+      </c>
+      <c r="G12" s="3">
+        <f>1-('lifetime scenario'!H11/baseline!F11)</f>
+        <v>4.2258251376362521E-3</v>
+      </c>
+      <c r="H12" s="3">
+        <f>1-('lifetime scenario'!I11/baseline!G11)</f>
+        <v>6.3501633588132211E-3</v>
+      </c>
+      <c r="I12" s="3">
+        <f>1-('lifetime scenario'!J11/baseline!H11)</f>
+        <v>7.4475455755842468E-3</v>
+      </c>
+      <c r="J12" s="3">
+        <f>1-('lifetime scenario'!K11/baseline!I11)</f>
+        <v>3.5585161586149106E-3</v>
+      </c>
+      <c r="K12" s="3">
+        <f>1-('lifetime scenario'!L11/baseline!J11)</f>
+        <v>4.4941068017805286E-3</v>
+      </c>
+      <c r="L12" s="3">
+        <f>1-('lifetime scenario'!M11/baseline!K11)</f>
+        <v>3.1641176170572605E-3</v>
+      </c>
+      <c r="N12" s="5">
+        <v>2033</v>
+      </c>
+      <c r="O12" s="3">
+        <f>1-SUM('lifetime scenario'!D11:M11)/SUM(baseline!B11:K11)</f>
+        <v>6.5284392862163809E-3</v>
+      </c>
+      <c r="R12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B13" s="5">
+        <v>2034</v>
+      </c>
+      <c r="C13" s="3">
+        <f>1-('lifetime scenario'!D12/baseline!B12)</f>
+        <v>1.5306196341571709E-2</v>
+      </c>
+      <c r="D13" s="3">
+        <f>1-('lifetime scenario'!E12/baseline!C12)</f>
+        <v>6.3291022805557207E-3</v>
+      </c>
+      <c r="E13" s="3">
+        <f>1-('lifetime scenario'!F12/baseline!D12)</f>
+        <v>6.3948928983051934E-3</v>
+      </c>
+      <c r="F13" s="3">
+        <f>1-('lifetime scenario'!G12/baseline!E12)</f>
+        <v>9.1460990803562403E-3</v>
+      </c>
+      <c r="G13" s="3">
+        <f>1-('lifetime scenario'!H12/baseline!F12)</f>
+        <v>6.152017996802206E-3</v>
+      </c>
+      <c r="H13" s="3">
+        <f>1-('lifetime scenario'!I12/baseline!G12)</f>
+        <v>9.4484661018483518E-3</v>
+      </c>
+      <c r="I13" s="3">
+        <f>1-('lifetime scenario'!J12/baseline!H12)</f>
+        <v>1.1124736632452947E-2</v>
+      </c>
+      <c r="J13" s="3">
+        <f>1-('lifetime scenario'!K12/baseline!I12)</f>
+        <v>5.5037524558311235E-3</v>
+      </c>
+      <c r="K13" s="3">
+        <f>1-('lifetime scenario'!L12/baseline!J12)</f>
+        <v>6.855318293650825E-3</v>
+      </c>
+      <c r="L13" s="3">
+        <f>1-('lifetime scenario'!M12/baseline!K12)</f>
+        <v>4.5788216087742084E-3</v>
+      </c>
+      <c r="N13" s="5">
+        <v>2034</v>
+      </c>
+      <c r="O13" s="3">
+        <f>1-SUM('lifetime scenario'!D12:M12)/SUM(baseline!B12:K12)</f>
+        <v>9.5463398675234012E-3</v>
+      </c>
+      <c r="R13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B14" s="5">
+        <v>2035</v>
+      </c>
+      <c r="C14" s="3">
+        <f>1-('lifetime scenario'!D13/baseline!B13)</f>
+        <v>2.111622523659773E-2</v>
+      </c>
+      <c r="D14" s="3">
+        <f>1-('lifetime scenario'!E13/baseline!C13)</f>
+        <v>9.2091048323449387E-3</v>
+      </c>
+      <c r="E14" s="3">
+        <f>1-('lifetime scenario'!F13/baseline!D13)</f>
+        <v>9.2584984402602766E-3</v>
+      </c>
+      <c r="F14" s="3">
+        <f>1-('lifetime scenario'!G13/baseline!E13)</f>
+        <v>1.2843268291777399E-2</v>
+      </c>
+      <c r="G14" s="3">
+        <f>1-('lifetime scenario'!H13/baseline!F13)</f>
+        <v>8.5291902294414301E-3</v>
+      </c>
+      <c r="H14" s="3">
+        <f>1-('lifetime scenario'!I13/baseline!G13)</f>
+        <v>1.3259614673816311E-2</v>
+      </c>
+      <c r="I14" s="3">
+        <f>1-('lifetime scenario'!J13/baseline!H13)</f>
+        <v>1.568866098518007E-2</v>
+      </c>
+      <c r="J14" s="3">
+        <f>1-('lifetime scenario'!K13/baseline!I13)</f>
+        <v>8.0950363803826697E-3</v>
+      </c>
+      <c r="K14" s="3">
+        <f>1-('lifetime scenario'!L13/baseline!J13)</f>
+        <v>9.9718118906351183E-3</v>
+      </c>
+      <c r="L14" s="3">
+        <f>1-('lifetime scenario'!M13/baseline!K13)</f>
+        <v>6.3567851778465467E-3</v>
+      </c>
+      <c r="N14" s="5">
+        <v>2035</v>
+      </c>
+      <c r="O14" s="3">
+        <f>1-SUM('lifetime scenario'!D13:M13)/SUM(baseline!B13:K13)</f>
+        <v>1.322158521410377E-2</v>
+      </c>
+      <c r="R14" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B15" s="5">
+        <v>2036</v>
+      </c>
+      <c r="C15" s="3">
+        <f>1-('lifetime scenario'!D14/baseline!B14)</f>
+        <v>2.7686903569292598E-2</v>
+      </c>
+      <c r="D15" s="3">
+        <f>1-('lifetime scenario'!E14/baseline!C14)</f>
+        <v>1.2867507482498874E-2</v>
+      </c>
+      <c r="E15" s="3">
+        <f>1-('lifetime scenario'!F14/baseline!D14)</f>
+        <v>1.2873351742698991E-2</v>
+      </c>
+      <c r="F15" s="3">
+        <f>1-('lifetime scenario'!G14/baseline!E14)</f>
+        <v>1.7262081831047271E-2</v>
+      </c>
+      <c r="G15" s="3">
+        <f>1-('lifetime scenario'!H14/baseline!F14)</f>
+        <v>1.1346190718058646E-2</v>
+      </c>
+      <c r="H15" s="3">
+        <f>1-('lifetime scenario'!I14/baseline!G14)</f>
+        <v>1.7710066703576E-2</v>
+      </c>
+      <c r="I15" s="3">
+        <f>1-('lifetime scenario'!J14/baseline!H14)</f>
+        <v>2.1033158812971631E-2</v>
+      </c>
+      <c r="J15" s="3">
+        <f>1-('lifetime scenario'!K14/baseline!I14)</f>
+        <v>1.1343335138398691E-2</v>
+      </c>
+      <c r="K15" s="3">
+        <f>1-('lifetime scenario'!L14/baseline!J14)</f>
+        <v>1.3882855486849421E-2</v>
+      </c>
+      <c r="L15" s="3">
+        <f>1-('lifetime scenario'!M14/baseline!K14)</f>
+        <v>8.5345452227089114E-3</v>
+      </c>
+      <c r="N15" s="5">
+        <v>2036</v>
+      </c>
+      <c r="O15" s="3">
+        <f>1-SUM('lifetime scenario'!D14:M14)/SUM(baseline!B14:K14)</f>
+        <v>1.7496715802307827E-2</v>
+      </c>
+      <c r="R15" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B16" s="5">
+        <v>2037</v>
+      </c>
+      <c r="C16" s="3">
+        <f>1-('lifetime scenario'!D15/baseline!B15)</f>
+        <v>3.4805979911090468E-2</v>
+      </c>
+      <c r="D16" s="3">
+        <f>1-('lifetime scenario'!E15/baseline!C15)</f>
+        <v>1.7319992447686228E-2</v>
+      </c>
+      <c r="E16" s="3">
+        <f>1-('lifetime scenario'!F15/baseline!D15)</f>
+        <v>1.7268702648153944E-2</v>
+      </c>
+      <c r="F16" s="3">
+        <f>1-('lifetime scenario'!G15/baseline!E15)</f>
+        <v>2.2338749167933436E-2</v>
+      </c>
+      <c r="G16" s="3">
+        <f>1-('lifetime scenario'!H15/baseline!F15)</f>
+        <v>1.4582003808965349E-2</v>
+      </c>
+      <c r="H16" s="3">
+        <f>1-('lifetime scenario'!I15/baseline!G15)</f>
+        <v>2.270227337034314E-2</v>
+      </c>
+      <c r="I16" s="3">
+        <f>1-('lifetime scenario'!J15/baseline!H15)</f>
+        <v>2.698689598846804E-2</v>
+      </c>
+      <c r="J16" s="3">
+        <f>1-('lifetime scenario'!K15/baseline!I15)</f>
+        <v>1.521082384661876E-2</v>
+      </c>
+      <c r="K16" s="3">
+        <f>1-('lifetime scenario'!L15/baseline!J15)</f>
+        <v>1.8617752897360562E-2</v>
+      </c>
+      <c r="L16" s="3">
+        <f>1-('lifetime scenario'!M15/baseline!K15)</f>
+        <v>1.1150615378390016E-2</v>
+      </c>
+      <c r="N16" s="5">
+        <v>2037</v>
+      </c>
+      <c r="O16" s="3">
+        <f>1-SUM('lifetime scenario'!D15:M15)/SUM(baseline!B15:K15)</f>
+        <v>2.2294729982710759E-2</v>
+      </c>
+      <c r="R16" s="11">
+        <f>1-(150/180)</f>
+        <v>0.16666666666666663</v>
+      </c>
+    </row>
+    <row r="17" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B17" s="5">
+        <v>2038</v>
+      </c>
+      <c r="C17" s="3">
+        <f>1-('lifetime scenario'!D16/baseline!B16)</f>
+        <v>4.2276016573017161E-2</v>
+      </c>
+      <c r="D17" s="3">
+        <f>1-('lifetime scenario'!E16/baseline!C16)</f>
+        <v>2.2567714851013276E-2</v>
+      </c>
+      <c r="E17" s="3">
+        <f>1-('lifetime scenario'!F16/baseline!D16)</f>
+        <v>2.2469402275238526E-2</v>
+      </c>
+      <c r="F17" s="3">
+        <f>1-('lifetime scenario'!G16/baseline!E16)</f>
+        <v>2.7981570043248083E-2</v>
+      </c>
+      <c r="G17" s="3">
+        <f>1-('lifetime scenario'!H16/baseline!F16)</f>
+        <v>1.8207371579610387E-2</v>
+      </c>
+      <c r="H17" s="3">
+        <f>1-('lifetime scenario'!I16/baseline!G16)</f>
+        <v>2.8114618317277906E-2</v>
+      </c>
+      <c r="I17" s="3">
+        <f>1-('lifetime scenario'!J16/baseline!H16)</f>
+        <v>3.3349243357090774E-2</v>
+      </c>
+      <c r="J17" s="3">
+        <f>1-('lifetime scenario'!K16/baseline!I16)</f>
+        <v>1.9596176625278128E-2</v>
+      </c>
+      <c r="K17" s="3">
+        <f>1-('lifetime scenario'!L16/baseline!J16)</f>
+        <v>2.4068415302398782E-2</v>
+      </c>
+      <c r="L17" s="3">
+        <f>1-('lifetime scenario'!M16/baseline!K16)</f>
+        <v>1.4230989764698831E-2</v>
+      </c>
+      <c r="N17" s="5">
+        <v>2038</v>
+      </c>
+      <c r="O17" s="3">
+        <f>1-SUM('lifetime scenario'!D16:M16)/SUM(baseline!B16:K16)</f>
+        <v>2.7538059144661897E-2</v>
+      </c>
+      <c r="R17" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B18" s="5">
+        <v>2039</v>
+      </c>
+      <c r="C18" s="3">
+        <f>1-('lifetime scenario'!D17/baseline!B17)</f>
+        <v>4.9995778040202943E-2</v>
+      </c>
+      <c r="D18" s="3">
+        <f>1-('lifetime scenario'!E17/baseline!C17)</f>
+        <v>2.8611393316903655E-2</v>
+      </c>
+      <c r="E18" s="3">
+        <f>1-('lifetime scenario'!F17/baseline!D17)</f>
+        <v>2.8489052741323961E-2</v>
+      </c>
+      <c r="F18" s="3">
+        <f>1-('lifetime scenario'!G17/baseline!E17)</f>
+        <v>3.4095529568312299E-2</v>
+      </c>
+      <c r="G18" s="3">
+        <f>1-('lifetime scenario'!H17/baseline!F17)</f>
+        <v>2.2185917043210934E-2</v>
+      </c>
+      <c r="H18" s="3">
+        <f>1-('lifetime scenario'!I17/baseline!G17)</f>
+        <v>3.3825551784410157E-2</v>
+      </c>
+      <c r="I18" s="3">
+        <f>1-('lifetime scenario'!J17/baseline!H17)</f>
+        <v>3.992437015547412E-2</v>
+      </c>
+      <c r="J18" s="3">
+        <f>1-('lifetime scenario'!K17/baseline!I17)</f>
+        <v>2.4363230556907811E-2</v>
+      </c>
+      <c r="K18" s="3">
+        <f>1-('lifetime scenario'!L17/baseline!J17)</f>
+        <v>3.0199957628625818E-2</v>
+      </c>
+      <c r="L18" s="3">
+        <f>1-('lifetime scenario'!M17/baseline!K17)</f>
+        <v>1.7764794787970439E-2</v>
+      </c>
+      <c r="N18" s="5">
+        <v>2039</v>
+      </c>
+      <c r="O18" s="3">
+        <f>1-SUM('lifetime scenario'!D17:M17)/SUM(baseline!B17:K17)</f>
+        <v>3.3165856039477748E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B19" s="5">
+        <v>2040</v>
+      </c>
+      <c r="C19" s="3">
+        <f>1-('lifetime scenario'!D18/baseline!B18)</f>
+        <v>5.7892065922594327E-2</v>
+      </c>
+      <c r="D19" s="3">
+        <f>1-('lifetime scenario'!E18/baseline!C18)</f>
+        <v>3.5385446773777418E-2</v>
+      </c>
+      <c r="E19" s="3">
+        <f>1-('lifetime scenario'!F18/baseline!D18)</f>
+        <v>3.5285293046378285E-2</v>
+      </c>
+      <c r="F19" s="3">
+        <f>1-('lifetime scenario'!G18/baseline!E18)</f>
+        <v>4.0567343126416855E-2</v>
+      </c>
+      <c r="G19" s="3">
+        <f>1-('lifetime scenario'!H18/baseline!F18)</f>
+        <v>2.6482279578080137E-2</v>
+      </c>
+      <c r="H19" s="3">
+        <f>1-('lifetime scenario'!I18/baseline!G18)</f>
+        <v>3.9716975354878725E-2</v>
+      </c>
+      <c r="I19" s="3">
+        <f>1-('lifetime scenario'!J18/baseline!H18)</f>
+        <v>4.6531584655267522E-2</v>
+      </c>
+      <c r="J19" s="3">
+        <f>1-('lifetime scenario'!K18/baseline!I18)</f>
+        <v>2.9369208210980657E-2</v>
+      </c>
+      <c r="K19" s="3">
+        <f>1-('lifetime scenario'!L18/baseline!J18)</f>
+        <v>3.6943112422986091E-2</v>
+      </c>
+      <c r="L19" s="3">
+        <f>1-('lifetime scenario'!M18/baseline!K18)</f>
+        <v>2.1701101209267049E-2</v>
+      </c>
+      <c r="N19" s="5">
+        <v>2040</v>
+      </c>
+      <c r="O19" s="3">
+        <f>1-SUM('lifetime scenario'!D18:M18)/SUM(baseline!B18:K18)</f>
+        <v>3.9106839655486669E-2</v>
+      </c>
+      <c r="R19" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="S19" s="12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B20" s="5">
+        <v>2041</v>
+      </c>
+      <c r="C20" s="3">
+        <f>1-('lifetime scenario'!D19/baseline!B19)</f>
+        <v>6.5896725830976499E-2</v>
+      </c>
+      <c r="D20" s="3">
+        <f>1-('lifetime scenario'!E19/baseline!C19)</f>
+        <v>4.2768109349485162E-2</v>
+      </c>
+      <c r="E20" s="3">
+        <f>1-('lifetime scenario'!F19/baseline!D19)</f>
+        <v>4.2800522099972649E-2</v>
+      </c>
+      <c r="F20" s="3">
+        <f>1-('lifetime scenario'!G19/baseline!E19)</f>
+        <v>4.7287046994108128E-2</v>
+      </c>
+      <c r="G20" s="3">
+        <f>1-('lifetime scenario'!H19/baseline!F19)</f>
+        <v>3.1050048523938445E-2</v>
+      </c>
+      <c r="H20" s="3">
+        <f>1-('lifetime scenario'!I19/baseline!G19)</f>
+        <v>4.5670407218381559E-2</v>
+      </c>
+      <c r="I20" s="3">
+        <f>1-('lifetime scenario'!J19/baseline!H19)</f>
+        <v>5.3045052907529477E-2</v>
+      </c>
+      <c r="J20" s="3">
+        <f>1-('lifetime scenario'!K19/baseline!I19)</f>
+        <v>3.4471836179149173E-2</v>
+      </c>
+      <c r="K20" s="3">
+        <f>1-('lifetime scenario'!L19/baseline!J19)</f>
+        <v>4.4138369917146592E-2</v>
+      </c>
+      <c r="L20" s="3">
+        <f>1-('lifetime scenario'!M19/baseline!K19)</f>
+        <v>2.5960069444556977E-2</v>
+      </c>
+      <c r="N20" s="5">
+        <v>2041</v>
+      </c>
+      <c r="O20" s="3">
+        <f>1-SUM('lifetime scenario'!D19:M19)/SUM(baseline!B19:K19)</f>
+        <v>4.5282458694226202E-2</v>
+      </c>
+      <c r="R20" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="S20" s="12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B21" s="5">
+        <v>2042</v>
+      </c>
+      <c r="C21" s="3">
+        <f>1-('lifetime scenario'!D20/baseline!B20)</f>
+        <v>7.3992933402045935E-2</v>
+      </c>
+      <c r="D21" s="3">
+        <f>1-('lifetime scenario'!E20/baseline!C20)</f>
+        <v>5.0642145560837015E-2</v>
+      </c>
+      <c r="E21" s="3">
+        <f>1-('lifetime scenario'!F20/baseline!D20)</f>
+        <v>5.1028838438303969E-2</v>
+      </c>
+      <c r="F21" s="3">
+        <f>1-('lifetime scenario'!G20/baseline!E20)</f>
+        <v>5.4135694564819259E-2</v>
+      </c>
+      <c r="G21" s="3">
+        <f>1-('lifetime scenario'!H20/baseline!F20)</f>
+        <v>3.5847938845624094E-2</v>
+      </c>
+      <c r="H21" s="3">
+        <f>1-('lifetime scenario'!I20/baseline!G20)</f>
+        <v>5.161572556291727E-2</v>
+      </c>
+      <c r="I21" s="3">
+        <f>1-('lifetime scenario'!J20/baseline!H20)</f>
+        <v>5.9417992738657666E-2</v>
+      </c>
+      <c r="J21" s="3">
+        <f>1-('lifetime scenario'!K20/baseline!I20)</f>
+        <v>3.9441571142859289E-2</v>
+      </c>
+      <c r="K21" s="3">
+        <f>1-('lifetime scenario'!L20/baseline!J20)</f>
+        <v>5.1704419167595272E-2</v>
+      </c>
+      <c r="L21" s="3">
+        <f>1-('lifetime scenario'!M20/baseline!K20)</f>
+        <v>3.0420536349779814E-2</v>
+      </c>
+      <c r="N21" s="5">
+        <v>2042</v>
+      </c>
+      <c r="O21" s="3">
+        <f>1-SUM('lifetime scenario'!D20:M20)/SUM(baseline!B20:K20)</f>
+        <v>5.1632239603470853E-2</v>
+      </c>
+      <c r="Q21" s="5">
+        <v>2019</v>
+      </c>
+      <c r="R21" s="3">
+        <f>R3</f>
+        <v>0</v>
+      </c>
+      <c r="S21" s="4">
+        <f>R21*$S$28/$R$28</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B22" s="5">
+        <v>2043</v>
+      </c>
+      <c r="C22" s="3">
+        <f>1-('lifetime scenario'!D21/baseline!B21)</f>
+        <v>8.2146455503790738E-2</v>
+      </c>
+      <c r="D22" s="3">
+        <f>1-('lifetime scenario'!E21/baseline!C21)</f>
+        <v>5.8965021730418621E-2</v>
+      </c>
+      <c r="E22" s="3">
+        <f>1-('lifetime scenario'!F21/baseline!D21)</f>
+        <v>5.9969349699053653E-2</v>
+      </c>
+      <c r="F22" s="3">
+        <f>1-('lifetime scenario'!G21/baseline!E21)</f>
+        <v>6.0988864539322729E-2</v>
+      </c>
+      <c r="G22" s="3">
+        <f>1-('lifetime scenario'!H21/baseline!F21)</f>
+        <v>4.0843363134360322E-2</v>
+      </c>
+      <c r="H22" s="3">
+        <f>1-('lifetime scenario'!I21/baseline!G21)</f>
+        <v>5.7475530071320002E-2</v>
+      </c>
+      <c r="I22" s="3">
+        <f>1-('lifetime scenario'!J21/baseline!H21)</f>
+        <v>6.5618500825156856E-2</v>
+      </c>
+      <c r="J22" s="3">
+        <f>1-('lifetime scenario'!K21/baseline!I21)</f>
+        <v>4.4164166032291563E-2</v>
+      </c>
+      <c r="K22" s="3">
+        <f>1-('lifetime scenario'!L21/baseline!J21)</f>
+        <v>5.9458192177478608E-2</v>
+      </c>
+      <c r="L22" s="3">
+        <f>1-('lifetime scenario'!M21/baseline!K21)</f>
+        <v>3.4943054618763569E-2</v>
+      </c>
+      <c r="N22" s="5">
+        <v>2043</v>
+      </c>
+      <c r="O22" s="3">
+        <f>1-SUM('lifetime scenario'!D21:M21)/SUM(baseline!B21:K21)</f>
+        <v>5.8098299615189974E-2</v>
+      </c>
+      <c r="Q22" s="5">
+        <v>2023</v>
+      </c>
+      <c r="R22" s="3">
+        <f t="shared" ref="R22:R28" si="0">R4</f>
+        <v>0</v>
+      </c>
+      <c r="S22" s="4">
+        <f t="shared" ref="S22:S27" si="1">R22*$S$28/$R$28</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B23" s="5">
+        <v>2044</v>
+      </c>
+      <c r="C23" s="3">
+        <f>1-('lifetime scenario'!D22/baseline!B22)</f>
+        <v>9.0396275506543611E-2</v>
+      </c>
+      <c r="D23" s="3">
+        <f>1-('lifetime scenario'!E22/baseline!C22)</f>
+        <v>6.7647293248147999E-2</v>
+      </c>
+      <c r="E23" s="3">
+        <f>1-('lifetime scenario'!F22/baseline!D22)</f>
+        <v>6.9459406606867113E-2</v>
+      </c>
+      <c r="F23" s="3">
+        <f>1-('lifetime scenario'!G22/baseline!E22)</f>
+        <v>6.7768866835101749E-2</v>
+      </c>
+      <c r="G23" s="3">
+        <f>1-('lifetime scenario'!H22/baseline!F22)</f>
+        <v>4.5995547373014256E-2</v>
+      </c>
+      <c r="H23" s="3">
+        <f>1-('lifetime scenario'!I22/baseline!G22)</f>
+        <v>6.3164423520476465E-2</v>
+      </c>
+      <c r="I23" s="3">
+        <f>1-('lifetime scenario'!J22/baseline!H22)</f>
+        <v>7.1651695027995288E-2</v>
+      </c>
+      <c r="J23" s="3">
+        <f>1-('lifetime scenario'!K22/baseline!I22)</f>
+        <v>4.8683202146339588E-2</v>
+      </c>
+      <c r="K23" s="3">
+        <f>1-('lifetime scenario'!L22/baseline!J22)</f>
+        <v>6.7382020241408269E-2</v>
+      </c>
+      <c r="L23" s="3">
+        <f>1-('lifetime scenario'!M22/baseline!K22)</f>
+        <v>3.9429635032045551E-2</v>
+      </c>
+      <c r="N23" s="5">
+        <v>2044</v>
+      </c>
+      <c r="O23" s="3">
+        <f>1-SUM('lifetime scenario'!D22:M22)/SUM(baseline!B22:K22)</f>
+        <v>6.4627882457843011E-2</v>
+      </c>
+      <c r="Q23" s="5">
+        <v>2025</v>
+      </c>
+      <c r="R23" s="3">
+        <f t="shared" si="0"/>
+        <v>8.856151468505935E-6</v>
+      </c>
+      <c r="S23" s="4">
+        <f t="shared" si="1"/>
+        <v>1.4322673269346312E-5</v>
+      </c>
+    </row>
+    <row r="24" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B24" s="5">
+        <v>2045</v>
+      </c>
+      <c r="C24" s="3">
+        <f>1-('lifetime scenario'!D23/baseline!B23)</f>
+        <v>9.8821622773929141E-2</v>
+      </c>
+      <c r="D24" s="3">
+        <f>1-('lifetime scenario'!E23/baseline!C23)</f>
+        <v>7.6453542165566657E-2</v>
+      </c>
+      <c r="E24" s="3">
+        <f>1-('lifetime scenario'!F23/baseline!D23)</f>
+        <v>7.9324128090259571E-2</v>
+      </c>
+      <c r="F24" s="3">
+        <f>1-('lifetime scenario'!G23/baseline!E23)</f>
+        <v>7.4411359132558919E-2</v>
+      </c>
+      <c r="G24" s="3">
+        <f>1-('lifetime scenario'!H23/baseline!F23)</f>
+        <v>5.127436584320666E-2</v>
+      </c>
+      <c r="H24" s="3">
+        <f>1-('lifetime scenario'!I23/baseline!G23)</f>
+        <v>6.8650174345507353E-2</v>
+      </c>
+      <c r="I24" s="3">
+        <f>1-('lifetime scenario'!J23/baseline!H23)</f>
+        <v>7.757317538997166E-2</v>
+      </c>
+      <c r="J24" s="3">
+        <f>1-('lifetime scenario'!K23/baseline!I23)</f>
+        <v>5.2981429766890797E-2</v>
+      </c>
+      <c r="K24" s="3">
+        <f>1-('lifetime scenario'!L23/baseline!J23)</f>
+        <v>7.5342727247264984E-2</v>
+      </c>
+      <c r="L24" s="3">
+        <f>1-('lifetime scenario'!M23/baseline!K23)</f>
+        <v>4.3821493102675024E-2</v>
+      </c>
+      <c r="N24" s="5">
+        <v>2045</v>
+      </c>
+      <c r="O24" s="3">
+        <f>1-SUM('lifetime scenario'!D23:M23)/SUM(baseline!B23:K23)</f>
+        <v>7.1177024926353694E-2</v>
+      </c>
+      <c r="Q24" s="5">
+        <v>2030</v>
+      </c>
+      <c r="R24" s="3">
+        <f t="shared" si="0"/>
+        <v>1.3763782578244399E-3</v>
+      </c>
+      <c r="S24" s="4">
+        <f t="shared" si="1"/>
+        <v>2.2259574208905526E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B25" s="5">
+        <v>2046</v>
+      </c>
+      <c r="C25" s="3">
+        <f>1-('lifetime scenario'!D24/baseline!B24)</f>
+        <v>0.10742777447579599</v>
+      </c>
+      <c r="D25" s="3">
+        <f>1-('lifetime scenario'!E24/baseline!C24)</f>
+        <v>8.534089709658399E-2</v>
+      </c>
+      <c r="E25" s="3">
+        <f>1-('lifetime scenario'!F24/baseline!D24)</f>
+        <v>8.9421156511447775E-2</v>
+      </c>
+      <c r="F25" s="3">
+        <f>1-('lifetime scenario'!G24/baseline!E24)</f>
+        <v>8.0893531307852706E-2</v>
+      </c>
+      <c r="G25" s="3">
+        <f>1-('lifetime scenario'!H24/baseline!F24)</f>
+        <v>5.6669726515601537E-2</v>
+      </c>
+      <c r="H25" s="3">
+        <f>1-('lifetime scenario'!I24/baseline!G24)</f>
+        <v>7.3940916758097885E-2</v>
+      </c>
+      <c r="I25" s="3">
+        <f>1-('lifetime scenario'!J24/baseline!H24)</f>
+        <v>8.3426433446237791E-2</v>
+      </c>
+      <c r="J25" s="3">
+        <f>1-('lifetime scenario'!K24/baseline!I24)</f>
+        <v>5.7042712303724263E-2</v>
+      </c>
+      <c r="K25" s="3">
+        <f>1-('lifetime scenario'!L24/baseline!J24)</f>
+        <v>8.3078287018196084E-2</v>
+      </c>
+      <c r="L25" s="3">
+        <f>1-('lifetime scenario'!M24/baseline!K24)</f>
+        <v>4.8079180672403132E-2</v>
+      </c>
+      <c r="N25" s="5">
+        <v>2046</v>
+      </c>
+      <c r="O25" s="3">
+        <f>1-SUM('lifetime scenario'!D24:M24)/SUM(baseline!B24:K24)</f>
+        <v>7.7714355884120234E-2</v>
+      </c>
+      <c r="Q25" s="5">
+        <v>2035</v>
+      </c>
+      <c r="R25" s="3">
+        <f t="shared" si="0"/>
+        <v>1.322158521410377E-2</v>
+      </c>
+      <c r="S25" s="4">
+        <f t="shared" si="1"/>
+        <v>2.1382701707153128E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B26" s="5">
+        <v>2047</v>
+      </c>
+      <c r="C26" s="3">
+        <f>1-('lifetime scenario'!D25/baseline!B25)</f>
+        <v>0.11609864321033092</v>
+      </c>
+      <c r="D26" s="3">
+        <f>1-('lifetime scenario'!E25/baseline!C25)</f>
+        <v>9.4128835797300026E-2</v>
+      </c>
+      <c r="E26" s="3">
+        <f>1-('lifetime scenario'!F25/baseline!D25)</f>
+        <v>9.9670597609726519E-2</v>
+      </c>
+      <c r="F26" s="3">
+        <f>1-('lifetime scenario'!G25/baseline!E25)</f>
+        <v>8.7202921388985777E-2</v>
+      </c>
+      <c r="G26" s="3">
+        <f>1-('lifetime scenario'!H25/baseline!F25)</f>
+        <v>6.2183459488452608E-2</v>
+      </c>
+      <c r="H26" s="3">
+        <f>1-('lifetime scenario'!I25/baseline!G25)</f>
+        <v>7.9122901836128912E-2</v>
+      </c>
+      <c r="I26" s="3">
+        <f>1-('lifetime scenario'!J25/baseline!H25)</f>
+        <v>8.9252900219292219E-2</v>
+      </c>
+      <c r="J26" s="3">
+        <f>1-('lifetime scenario'!K25/baseline!I25)</f>
+        <v>6.0878177414920187E-2</v>
+      </c>
+      <c r="K26" s="3">
+        <f>1-('lifetime scenario'!L25/baseline!J25)</f>
+        <v>9.0498779892504877E-2</v>
+      </c>
+      <c r="L26" s="3">
+        <f>1-('lifetime scenario'!M25/baseline!K25)</f>
+        <v>5.2219626323058987E-2</v>
+      </c>
+      <c r="N26" s="5">
+        <v>2047</v>
+      </c>
+      <c r="O26" s="3">
+        <f>1-SUM('lifetime scenario'!D25:M25)/SUM(baseline!B25:K25)</f>
+        <v>8.4200271548861449E-2</v>
+      </c>
+      <c r="Q26" s="5">
+        <v>2040</v>
+      </c>
+      <c r="R26" s="3">
+        <f t="shared" si="0"/>
+        <v>3.9106839655486669E-2</v>
+      </c>
+      <c r="S26" s="4">
+        <f t="shared" si="1"/>
+        <v>6.3245811566583862E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B27" s="5">
+        <v>2048</v>
+      </c>
+      <c r="C27" s="3">
+        <f>1-('lifetime scenario'!D26/baseline!B26)</f>
+        <v>0.12482085039723723</v>
+      </c>
+      <c r="D27" s="3">
+        <f>1-('lifetime scenario'!E26/baseline!C26)</f>
+        <v>0.10270446444008885</v>
+      </c>
+      <c r="E27" s="3">
+        <f>1-('lifetime scenario'!F26/baseline!D26)</f>
+        <v>0.10997664496042281</v>
+      </c>
+      <c r="F27" s="3">
+        <f>1-('lifetime scenario'!G26/baseline!E26)</f>
+        <v>9.3400597751186032E-2</v>
+      </c>
+      <c r="G27" s="3">
+        <f>1-('lifetime scenario'!H26/baseline!F26)</f>
+        <v>6.7805359587621017E-2</v>
+      </c>
+      <c r="H27" s="3">
+        <f>1-('lifetime scenario'!I26/baseline!G26)</f>
+        <v>8.427964517701525E-2</v>
+      </c>
+      <c r="I27" s="3">
+        <f>1-('lifetime scenario'!J26/baseline!H26)</f>
+        <v>9.5117362709155828E-2</v>
+      </c>
+      <c r="J27" s="3">
+        <f>1-('lifetime scenario'!K26/baseline!I26)</f>
+        <v>6.4607236533687495E-2</v>
+      </c>
+      <c r="K27" s="3">
+        <f>1-('lifetime scenario'!L26/baseline!J26)</f>
+        <v>9.7560553373145509E-2</v>
+      </c>
+      <c r="L27" s="3">
+        <f>1-('lifetime scenario'!M26/baseline!K26)</f>
+        <v>5.6285963569185138E-2</v>
+      </c>
+      <c r="N27" s="5">
+        <v>2048</v>
+      </c>
+      <c r="O27" s="3">
+        <f>1-SUM('lifetime scenario'!D26:M26)/SUM(baseline!B26:K26)</f>
+        <v>9.0625722986076518E-2</v>
+      </c>
+      <c r="Q27" s="5">
+        <v>2045</v>
+      </c>
+      <c r="R27" s="3">
+        <f t="shared" si="0"/>
+        <v>7.1177024926353694E-2</v>
+      </c>
+      <c r="S27" s="4">
+        <f t="shared" si="1"/>
+        <v>0.11511154432369554</v>
+      </c>
+    </row>
+    <row r="28" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B28" s="5">
+        <v>2049</v>
+      </c>
+      <c r="C28" s="3">
+        <f>1-('lifetime scenario'!D27/baseline!B27)</f>
+        <v>0.13358915147432238</v>
+      </c>
+      <c r="D28" s="3">
+        <f>1-('lifetime scenario'!E27/baseline!C27)</f>
+        <v>0.11109334463032472</v>
+      </c>
+      <c r="E28" s="3">
+        <f>1-('lifetime scenario'!F27/baseline!D27)</f>
+        <v>0.12019555530216974</v>
+      </c>
+      <c r="F28" s="3">
+        <f>1-('lifetime scenario'!G27/baseline!E27)</f>
+        <v>9.9549014767928656E-2</v>
+      </c>
+      <c r="G28" s="3">
+        <f>1-('lifetime scenario'!H27/baseline!F27)</f>
+        <v>7.3525088275124051E-2</v>
+      </c>
+      <c r="H28" s="3">
+        <f>1-('lifetime scenario'!I27/baseline!G27)</f>
+        <v>8.9458932531772062E-2</v>
+      </c>
+      <c r="I28" s="3">
+        <f>1-('lifetime scenario'!J27/baseline!H27)</f>
+        <v>0.1010918808910537</v>
+      </c>
+      <c r="J28" s="3">
+        <f>1-('lifetime scenario'!K27/baseline!I27)</f>
+        <v>6.8390602051042748E-2</v>
+      </c>
+      <c r="K28" s="3">
+        <f>1-('lifetime scenario'!L27/baseline!J27)</f>
+        <v>0.10429592135838051</v>
+      </c>
+      <c r="L28" s="3">
+        <f>1-('lifetime scenario'!M27/baseline!K27)</f>
+        <v>6.0334021571742946E-2</v>
+      </c>
+      <c r="N28" s="5">
+        <v>2049</v>
+      </c>
+      <c r="O28" s="3">
+        <f>1-SUM('lifetime scenario'!D27:M27)/SUM(baseline!B27:K27)</f>
+        <v>9.6991843160683211E-2</v>
+      </c>
+      <c r="Q28" s="7">
+        <v>2050</v>
+      </c>
+      <c r="R28" s="3">
+        <f t="shared" si="0"/>
+        <v>0.10326126048032036</v>
+      </c>
+      <c r="S28" s="4">
+        <v>0.16700000000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B29" s="5">
+        <v>2050</v>
+      </c>
+      <c r="C29" s="3">
+        <f>1-('lifetime scenario'!D28/baseline!B28)</f>
+        <v>0.14223958477370313</v>
+      </c>
+      <c r="D29" s="3">
+        <f>1-('lifetime scenario'!E28/baseline!C28)</f>
+        <v>0.11909343380814053</v>
+      </c>
+      <c r="E29" s="3">
+        <f>1-('lifetime scenario'!F28/baseline!D28)</f>
+        <v>0.13015387249286636</v>
+      </c>
+      <c r="F29" s="3">
+        <f>1-('lifetime scenario'!G28/baseline!E28)</f>
+        <v>0.10559852752733989</v>
+      </c>
+      <c r="G29" s="3">
+        <f>1-('lifetime scenario'!H28/baseline!F28)</f>
+        <v>7.9345025226425392E-2</v>
+      </c>
+      <c r="H29" s="3">
+        <f>1-('lifetime scenario'!I28/baseline!G28)</f>
+        <v>9.4627396376015138E-2</v>
+      </c>
+      <c r="I29" s="3">
+        <f>1-('lifetime scenario'!J28/baseline!H28)</f>
+        <v>0.10716745978755349</v>
+      </c>
+      <c r="J29" s="3">
+        <f>1-('lifetime scenario'!K28/baseline!I28)</f>
+        <v>7.2330974022021155E-2</v>
+      </c>
+      <c r="K29" s="3">
+        <f>1-('lifetime scenario'!L28/baseline!J28)</f>
+        <v>0.11057997785644336</v>
+      </c>
+      <c r="L29" s="3">
+        <f>1-('lifetime scenario'!M28/baseline!K28)</f>
+        <v>6.4469801774596158E-2</v>
+      </c>
+      <c r="N29" s="5">
+        <v>2050</v>
+      </c>
+      <c r="O29" s="3">
+        <f>1-SUM('lifetime scenario'!D28:M28)/SUM(baseline!B28:K28)</f>
+        <v>0.10326126048032036</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="R14" r:id="rId1" xr:uid="{56A34335-C361-487A-A3FD-E3A152610B90}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>